<commit_message>
feat(quotation): pre-fill 人天 to hit NT$200,000 一次性 total
Each Phase A/B/C line item now has a suggested 人天 in the source
list (3/4/3 split, fractional 0.5 where appropriate). The total
lands at 10 人天 × NT$20,000 = NT$200,000 untaxed = NT$210,000
including 5% VAT.

Distribution rationale:
- Phase A (3 人天): basic infra, lean cloud setup
- Phase B (4 人天): core conversation flow — the meat of POC
- Phase C (3 人天): advanced features bundled tight for a 4-6
  week timeline; 0.5 per item signals 'POC slice' scope

To change the total: edit the third tuple value on each phase
list in scripts/build_quotation.py and re-run; everything else
auto-updates.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/POC_報價單_杰隆印刷.xlsx
+++ b/POC_報價單_杰隆印刷.xlsx
@@ -16,8 +16,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="&quot;NT$&quot; #,##0"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="0.0"/>
+    <numFmt numFmtId="165" formatCode="&quot;NT$&quot; #,##0"/>
   </numFmts>
   <fonts count="14">
     <font>
@@ -152,13 +153,13 @@
     <xf numFmtId="0" fontId="7" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -167,11 +168,11 @@
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="12" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="12" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -694,7 +695,9 @@
           <t>GCP / AWS 帳號設定、VPC、IAM、Secret 管理</t>
         </is>
       </c>
-      <c r="C14" s="8" t="n"/>
+      <c r="C14" s="8" t="n">
+        <v>0.5</v>
+      </c>
       <c r="D14" s="9" t="n">
         <v>20000</v>
       </c>
@@ -714,7 +717,9 @@
           <t>訂單草稿 / 客戶 / 對話紀錄 / 知識庫 schema</t>
         </is>
       </c>
-      <c r="C15" s="8" t="n"/>
+      <c r="C15" s="8" t="n">
+        <v>1</v>
+      </c>
       <c r="D15" s="9" t="n">
         <v>20000</v>
       </c>
@@ -734,7 +739,9 @@
           <t>後端服務容器化、反向代理、TLS 設定</t>
         </is>
       </c>
-      <c r="C16" s="8" t="n"/>
+      <c r="C16" s="8" t="n">
+        <v>1</v>
+      </c>
       <c r="D16" s="9" t="n">
         <v>20000</v>
       </c>
@@ -754,7 +761,9 @@
           <t>GitHub Actions、Log/Error 監控初始化</t>
         </is>
       </c>
-      <c r="C17" s="8" t="n"/>
+      <c r="C17" s="8" t="n">
+        <v>0.5</v>
+      </c>
       <c r="D17" s="9" t="n">
         <v>20000</v>
       </c>
@@ -792,7 +801,9 @@
           <t>接單主流程、條件分支、轉接邏輯（於 Odin Studio 內設計）</t>
         </is>
       </c>
-      <c r="C20" s="8" t="n"/>
+      <c r="C20" s="8" t="n">
+        <v>1</v>
+      </c>
       <c r="D20" s="9" t="n">
         <v>20000</v>
       </c>
@@ -812,7 +823,9 @@
           <t>LLM Prompt 工程、欄位缺口偵測、白話追問生成</t>
         </is>
       </c>
-      <c r="C21" s="8" t="n"/>
+      <c r="C21" s="8" t="n">
+        <v>1</v>
+      </c>
       <c r="D21" s="9" t="n">
         <v>20000</v>
       </c>
@@ -832,7 +845,9 @@
           <t>嵌入式對話框、訊息流、模擬圖預覽元件</t>
         </is>
       </c>
-      <c r="C22" s="8" t="n"/>
+      <c r="C22" s="8" t="n">
+        <v>1</v>
+      </c>
       <c r="D22" s="9" t="n">
         <v>20000</v>
       </c>
@@ -852,7 +867,9 @@
           <t>Session 持久化、訂單 JSON schema、後端 API</t>
         </is>
       </c>
-      <c r="C23" s="8" t="n"/>
+      <c r="C23" s="8" t="n">
+        <v>1</v>
+      </c>
       <c r="D23" s="9" t="n">
         <v>20000</v>
       </c>
@@ -890,7 +907,9 @@
           <t>LLM Vision 串接、設計稿色數與尺寸建議</t>
         </is>
       </c>
-      <c r="C26" s="8" t="n"/>
+      <c r="C26" s="8" t="n">
+        <v>0.5</v>
+      </c>
       <c r="D26" s="9" t="n">
         <v>20000</v>
       </c>
@@ -910,7 +929,9 @@
           <t>Image Gen API 串接、貼標情境圖輸出</t>
         </is>
       </c>
-      <c r="C27" s="8" t="n"/>
+      <c r="C27" s="8" t="n">
+        <v>0.5</v>
+      </c>
       <c r="D27" s="9" t="n">
         <v>20000</v>
       </c>
@@ -930,7 +951,9 @@
           <t>Email / 電話比對、歷史訂單帶入流程</t>
         </is>
       </c>
-      <c r="C28" s="8" t="n"/>
+      <c r="C28" s="8" t="n">
+        <v>0.5</v>
+      </c>
       <c r="D28" s="9" t="n">
         <v>20000</v>
       </c>
@@ -950,7 +973,9 @@
           <t>情緒分類、Email / LINE Webhook 通知</t>
         </is>
       </c>
-      <c r="C29" s="8" t="n"/>
+      <c r="C29" s="8" t="n">
+        <v>0.5</v>
+      </c>
       <c r="D29" s="9" t="n">
         <v>20000</v>
       </c>
@@ -970,7 +995,9 @@
           <t>Bug 修正、上線切換、煙霧測試</t>
         </is>
       </c>
-      <c r="C30" s="8" t="n"/>
+      <c r="C30" s="8" t="n">
+        <v>0.5</v>
+      </c>
       <c r="D30" s="9" t="n">
         <v>20000</v>
       </c>
@@ -990,7 +1017,9 @@
           <t>業務操作訓練（1 小時）、技術交接文件</t>
         </is>
       </c>
-      <c r="C31" s="8" t="n"/>
+      <c r="C31" s="8" t="n">
+        <v>0.5</v>
+      </c>
       <c r="D31" s="9" t="n">
         <v>20000</v>
       </c>

</xml_diff>